<commit_message>
Recovered Actual Output values from original files because external API is currently down
</commit_message>
<xml_diff>
--- a/IT23183940_Assignment 1 - Test cases.xlsx
+++ b/IT23183940_Assignment 1 - Test cases.xlsx
@@ -521,7 +521,11 @@
           <t>ඔයාගේ බර්ත්ඩේ එක කවදාද කියලා දන්නවාද?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ඔයාගෙ birthday එක කවදාද කියලා දන්නවාද?</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -559,7 +563,11 @@
           <t>ඔයා හරි වෙලාවට ආවේ නේද? කොහොමද trip එක?</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ඔයා හරි වෙලාවට ආවෙ නේද? කොහොමද trip එක?</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -597,7 +605,11 @@
           <t>වහාම යනවා, නැත්නම් late වෙනවා.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>වහාම යනවා, නත්තම් late වෙනවා.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -635,7 +647,11 @@
           <t>වැඩ කරලා ඉවරම මැසේජ් එකක් දාන්නකෝ</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>වෙද krl ඉවරම් msg එක්ක් දන්නකො</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -673,7 +689,11 @@
           <t>සුභ අලුත් අවුරුද්දක් වේවා මචං!</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>සුබ අලුත් අවුරුද්දක් වෙවා මචන්!</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -711,7 +731,11 @@
           <t>මචන් බොහොම කාලකින්! කොහොමද ඔයා දැන්?</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>මචං බොහොම කාලකින්! කොහොමද ඔයා දැන්?</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -749,7 +773,11 @@
           <t>කරුණාකරලා මගේ bag එක පොඩ්ඩක් බලාහින්න.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>කරුණාකරලා මගේ බග් එක පොඩ්ඩක් බලහින්න.</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -787,7 +815,11 @@
           <t>අපි එක්ක යනවා නම් මාමත් එවන්න. මේක පොඩ්ඩක් බලන්න පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>අපි එක්ක යනවා නම් මමත් එවන්න. මේක පොඩ්ඩක් බලන්න පුළුවන්ද?</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -825,7 +857,11 @@
           <t>නෑ, මම දන්නේ නෑ ඒක.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>නැහැ, මම දන්නේ නැහැ ඒක.</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -863,7 +899,11 @@
           <t>අයියෝ, ඒක වගේ වුනොත් අමාරු තමයි මචන්.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>අයියො, එක වගෙ උනොත් අමාරු තමයි මචන්.</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -901,7 +941,11 @@
           <t>මාර මාර වැඩ තමයි මේ දවස් වල වෙන්නේ</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>මර මර වෙද තමා මෙ dws wl වෙන්නෙ</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -939,7 +983,11 @@
           <t>හෙමින් හෙමින් යමන් තියෙනවා තමයි වෙලා</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>හෙමින් හෙමින් යම්න් tynwa තමා වෙලා</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -977,7 +1025,11 @@
           <t>අඩෝ!!!! මොකක්ද ඒ සීන් එක....??</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>අඩො!!!! මොක්ක්ද් එ සෙඑන් එක....??</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1015,7 +1067,11 @@
           <t>මම යනවා, ඔයාත් එන්නේ නේද මචං පස්සේ?</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>මම යනවා, ඔයත් එන්න නේද මචං පස්සේ?</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1053,7 +1109,11 @@
           <t>මාමත් එන්නම් මචංග්.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>මමත් එන්නම් මචන්.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1091,7 +1151,11 @@
           <t>ඔයාට පුළුවන් නම් ඒක කරන්න. මම හෙට එවන්නම්.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ඔයාට පුළුවන් නම් ඒක කරන්න. මම හෙට එවන්ම්.</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1129,7 +1193,11 @@
           <t>අපි අද බත් සහ ව්‍යංජන ගන්න ගියා කැන්ටිමට.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>අපි අද rice and curry ගන්න ගියා canteen එකට.</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1167,7 +1235,11 @@
           <t>ඔයා දන්නවද නව movie එකේ trailer එක release උනා කියලා?</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ඔයා දන්නවද නව movie එකේ trailer එක release වුණා කියලා?</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1205,7 +1277,11 @@
           <t>මට අවුට් ඔෆ් ද බොක්ස් හිතන්න ඕනේ මේකට.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>මට out of the box හිතන්න ඔනෙ මෙකට.</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1243,7 +1319,11 @@
           <t>මචන් අපි ළඟදීම හමුවිය යුතුයි, ගොඩක් කාලෙකින්.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>මචන් we should catch up soon, ගොඩක් කාලකින්.</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1281,7 +1361,11 @@
           <t>ඔයාගේ laptop එකේ RAM කොච්චරද?</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ඔයාගෙ laptop එකේ RAM කොච්චරද?</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1319,7 +1403,11 @@
           <t>මගේ පරිගණකයේ තිරය බෙදාගන්න පුළුවන්ද මීටින් එකේ?</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>මගෙ PC එකෙ screenshare කරන්න පුලුවන්ද meeting එකෙ?</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1357,7 +1445,11 @@
           <t>YouTube එකේ subscribe කරන්න, TikTok එකේ follow කරන්න.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>YouTube ඒකේ subscribe කරන්න, TikTok එකේ follow කරන්න.</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1395,7 +1487,11 @@
           <t>ඉන්ස්ටග්‍රෑම් ස්ටෝරි එක පෝස්ට් කරපන්. ෆේස්බුක් එකටත් ශෙයාර් කරපන්.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Instagram story එක post කරපන්. Facebook එකටත් share කරපන්.</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1435,7 +1531,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>මම යනවා, ඔයත් එන්න නේද මචං පස්සේ?</t>
+          <t>DOB එක submit කරන්ඩ පෙන්නන්න.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1475,9 +1571,14 @@
           <t>මානව සම්පත් අංශය කිව්වා ජීව දත්ත සටහන පීඩීඑෆ් විදිහට එවන්න කියලා. හැකි ඉක්මනින් එවන්න.</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>HR කිව්වා CV එක PDF විදිහට එවන්න කියලා. ASAP එවන්න.</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1512,9 +1613,14 @@
           <t>අපේ මහාචාර්යතුමා කිව්වා හෙට විද්‍යාගාරය අවලංගුයි කියලා.</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>අපෙ prof කිව්වා හෙට lab එක cancel කියලා.</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1549,9 +1655,14 @@
           <t>අපේ prof කිව්වා assignment එක sub කරන්න deadline extend කියලා.</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>අපේ prof කිව assignment එක sub කරන්න deadline extend කියලා.</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1586,9 +1697,14 @@
           <t>මාතර වලට යනවා, Mirissa beach එකටත් යමුද?</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>මාතර වලට යනවා, මිරිස්ස beach එකටත් යමුද?</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1623,9 +1739,14 @@
           <t>නුගේගොඩ හන්දියට එන්න, මහරගමට පස්සේ.</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Nugegoda junction වලට එන්න, Maharagama පස්සෙ.</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1660,9 +1781,14 @@
           <t>කසුන් කිව්වා මම යනවා කියලා.</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>කසුන් කිවා මම යනවා කියලා.</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1697,9 +1823,14 @@
           <t>නිමේෂා සහ දිනෙත් දෙන්නා අම්මා එක්ක පන්තියේ ඉන්නවා.</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Nimasha සහ Dineth දෙන්නා ama එක්ක class එකෙ ඉන්නවා.</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1734,9 +1865,14 @@
           <t>අපි 3rd attempt එකේ pass උනා.</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>අපි 3rd attempt එකේ pass වුණා.</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1771,9 +1907,14 @@
           <t>10වෙනි දවසෙත් ආවේ නැති උනාම කොහොමද.</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>10weni දවසෙත් ආවෙ නති උනම කොහොමද.</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1808,9 +1949,14 @@
           <t>මට Rs.1000 දෙන්න පුළුවන්ද මචං?</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>මට Rs.1000 දෙන්න පුළුවන් ද මචන්?</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1845,9 +1991,14 @@
           <t>ෆෝන් එක පවුම් දෙසිය අනූනවයකින් ගත්තා තීරු බදු රහිතව.</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>phone එක GBP 299 වලින් ගත්තා duty free එකෙන්.</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1882,9 +2033,14 @@
           <t>meeting එක 9:00AM start වෙනවා.</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>meeting එක 9:00AM ස්ටාර්ට් වෙනවා.</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1919,9 +2075,14 @@
           <t>හෙට 6:00AM වලට නඟිනවා, 11:30PM වලට නිදාගන්නම්.</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>හෙට 6:00AM වලට නතනවා, 11:30PM වලට නිදාගන්නම්.</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1956,7 +2117,11 @@
           <t>උත්සවය මැයි පහට. ජුනි දහය වෙනකන් ලියාපදිංචි වෙන්න.</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>event එක May 5 වලට. June 10 වෙනකන් register කරන්න.</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1994,7 +2159,11 @@
           <t>මාර්තු තිස්එක වෙනකන් කරනවා. අප්‍රේල් එකට අලුත් යාවත්කාලීන කිරීම.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>March 31 වෙනකන් කරනා. April 1 වලට new update එක.</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2032,7 +2201,11 @@
           <t>ඒ ගසේ උස feet 20 විතර වෙනවා.</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ඒ ගසේ උස ෆීට්ස් 20 විතර වෙනවා.</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2070,7 +2243,11 @@
           <t>මම හෙට කිලෝමීටර් පහක් දුවන්න හිතන් ඉන්නේ. විතර විනාඩි හතළිස් පහක් යයි.</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>මම හෙට km 5k run කරන්න හිතන් ඉන්නෙ. විතර 45 minutes ලගයි.</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2108,7 +2285,11 @@
           <t>අඩෝ මේක ගොඩක් මාර scene එකක්. සෙට් තමයි bro.</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>අඩෝ මේක ගොඩක් මාර scene එකක්. set තමයි bro.</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2146,7 +2327,11 @@
           <t>මචං උඹ ගොඩක් නියමයි. මේක හොඳට හදලා.</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>මචන්ග් උබ ගොඩක් නියමයි. මෙක හොදට හදලා.</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2184,7 +2369,11 @@
           <t>නව blog එක බලන්න: www.islandlife.lk/travel කියලා.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>නව බ්ලොග් එක බලන්න: www.islandlife.lk/travel කියලා.</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2222,7 +2411,11 @@
           <t>මට test@gmail.com මේල් එකක් දාන්න.</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>මට test@gmail.com mail එකක් දාන්න.</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2260,7 +2453,11 @@
           <t>හාහා මේක නියාමයි 😂</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>හාහා මේක නියමයි 😂</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2298,7 +2495,11 @@
           <t>අඩෝ අද මාර බොරුවක් උනේ මට 😤 මම එයාව මාර විදිහට trust කළා.</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>අඩෝ අද මාර බොරුවක් උනේ මට  මම එයාව මාර විදිහට trust කරා.</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2338,7 +2539,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>event එක May 5 වලට. ජූනි 10 වෙනකන් register කරන්න.</t>
+          <t>අම්මො එක නම් සිරාවටම.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2378,9 +2579,14 @@
           <t>මචං හෙට 9:00AM වලට interview එකක් තියෙනවා. bus එකෙන් යනවා නිසා පොඩ්ඩක් late වෙනවා. සාචිනි කිව්වා outfit එක smart විදිහට select කරන්න. wish me luck!</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>මචං හෙට 9:00AM වලට interview එකක් තියෙනවා. බස් එකෙන් යනවා නිසා පොඩ්ඩක් late වෙනවා. සචිනි කිව outfit එක smart විදිහට select කරන්න. wish me luck!</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">

</xml_diff>